<commit_message>
Add Excel file input and update Excel tempelate
</commit_message>
<xml_diff>
--- a/example/Excel Template for HWTT.xlsx
+++ b/example/Excel Template for HWTT.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usdot-my.sharepoint.com/personal/farhad_abdollahi_ctr_ad_dot_gov/Documents/GitHub_HWTT_Analysis_Tool/HWTT_Analysis_Tool/example/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BD69BDA0-91AA-41A6-AFBF-747FADBB4C07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="40" documentId="8_{BD69BDA0-91AA-41A6-AFBF-747FADBB4C07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FDEAD05F-A961-448D-A40D-193EAF34B7DA}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{70AE326B-37D4-4DA4-87DA-F5BA518FA4A0}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{70AE326B-37D4-4DA4-87DA-F5BA518FA4A0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,23 +36,14 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="24">
-  <si>
-    <t>Passes - left wheel</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="26">
   <si>
     <t>Rut depth (mm)</t>
   </si>
   <si>
-    <t>Passes - right wheel</t>
-  </si>
-  <si>
     <t>Testing condition</t>
   </si>
   <si>
-    <t>Wet</t>
-  </si>
-  <si>
     <t>Parameter</t>
   </si>
   <si>
@@ -74,9 +65,6 @@
     <t>Project</t>
   </si>
   <si>
-    <t>-</t>
-  </si>
-  <si>
     <t>Project name</t>
   </si>
   <si>
@@ -92,22 +80,40 @@
     <t>Comment on the material</t>
   </si>
   <si>
-    <t>Sampling Time</t>
-  </si>
-  <si>
-    <t>Testing Time</t>
-  </si>
-  <si>
-    <t>Date and time of testing</t>
-  </si>
-  <si>
-    <t>Date and time of sample collection/preparation</t>
-  </si>
-  <si>
     <t>Technician name</t>
   </si>
   <si>
     <t xml:space="preserve">Name of the technician operating the test. </t>
+  </si>
+  <si>
+    <t>…</t>
+  </si>
+  <si>
+    <t>FD</t>
+  </si>
+  <si>
+    <t>Test Time</t>
+  </si>
+  <si>
+    <t>Test Date</t>
+  </si>
+  <si>
+    <t>Date of testing</t>
+  </si>
+  <si>
+    <t>Time of testing</t>
+  </si>
+  <si>
+    <t>Passes</t>
+  </si>
+  <si>
+    <t>Temperature (°C)</t>
+  </si>
+  <si>
+    <t>Wheather the left or right side of HWTT was used</t>
+  </si>
+  <si>
+    <t>Wheel Side</t>
   </si>
 </sst>
 </file>
@@ -252,7 +258,54 @@
       <right style="thin">
         <color indexed="64"/>
       </right>
-      <top/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
@@ -265,7 +318,9 @@
       <right style="thin">
         <color indexed="64"/>
       </right>
-      <top/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
@@ -278,53 +333,10 @@
       <right style="medium">
         <color indexed="64"/>
       </right>
-      <top/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
       <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -333,25 +345,39 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -368,6 +394,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -667,122 +697,163 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{65BE9D2A-A675-429C-92C5-A774EA04E6BF}">
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="22.85546875" style="14" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.42578125" style="14" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.28515625" style="14" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.42578125" style="14" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="23.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="27.28515625" customWidth="1"/>
-    <col min="8" max="8" width="48.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.85546875" style="9" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.85546875" style="9" customWidth="1"/>
+    <col min="3" max="3" width="21.140625" style="9" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="27.28515625" customWidth="1"/>
+    <col min="7" max="7" width="48.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="13" t="s">
+    <row r="1" spans="1:7" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="B1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="C1" s="8" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E2" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G2" s="7" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E3" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="13" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="13" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F2" s="10" t="s">
+      <c r="F3" s="14"/>
+      <c r="G3" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="G2" s="11" t="s">
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H2" s="12" t="s">
+      <c r="F4" s="10">
+        <v>50</v>
+      </c>
+      <c r="G4" s="2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="F3" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="G3" s="8" t="s">
-        <v>4</v>
-      </c>
-      <c r="H3" s="9" t="s">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E5" s="16" t="s">
+        <v>25</v>
+      </c>
+      <c r="F5" s="18"/>
+      <c r="G5" s="17" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E6" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="F4" s="2" t="s">
+      <c r="F6" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="G6" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="G4" s="1">
-        <v>50</v>
-      </c>
-      <c r="H4" s="3" t="s">
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E7" s="1" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="F5" s="2" t="s">
+      <c r="F7" s="9"/>
+      <c r="G7" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G5" s="1" t="s">
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E8" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="H5" s="3" t="s">
+      <c r="F8" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="G8" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="F6" s="2" t="s">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E9" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="F9" s="12">
+        <v>0.70833333333333337</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E10" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F10" s="9"/>
+      <c r="G10" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E11" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="G6" s="1"/>
-      <c r="H6" s="3" t="s">
+      <c r="F11" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="G11" s="4" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="F7" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="G7" s="1"/>
-      <c r="H7" s="3" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="F8" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G8" s="1"/>
-      <c r="H8" s="3" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="F9" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="G9" s="1"/>
-      <c r="H9" s="3" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F10" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="G10" s="5"/>
-      <c r="H10" s="6" t="s">
-        <v>23</v>
-      </c>
-    </row>
   </sheetData>
+  <dataValidations count="8">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A2:B1048576" xr:uid="{F3E1C8F5-DFCB-47CA-9E45-854ACBC499F4}">
+      <formula1>0</formula1>
+      <formula2>999999</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C1048576" xr:uid="{4AFCC87C-1028-4409-BFCB-20E8CCCD25F3}">
+      <formula1>0</formula1>
+      <formula2>999</formula2>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F3" xr:uid="{F60BFF27-73F4-457B-8100-F1AD200C7A78}">
+      <formula1>"Wet,Dry"</formula1>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F4" xr:uid="{1FBA003B-7F8E-4FFF-BEF1-24B84FE9DF39}">
+      <formula1>0</formula1>
+      <formula2>99</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F7" xr:uid="{384A6D86-B099-48EC-ADDF-1DDD4B24DFDB}">
+      <formula1>1000</formula1>
+      <formula2>99999</formula2>
+    </dataValidation>
+    <dataValidation type="time" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F9" xr:uid="{D355D9EE-48B0-4C39-A2F6-2217C4421456}">
+      <formula1>0</formula1>
+      <formula2>0.999305555555556</formula2>
+    </dataValidation>
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F10" xr:uid="{FA9112A1-20CC-40A9-9477-C78D48D200DC}">
+      <formula1>1</formula1>
+      <formula2>73050</formula2>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F5" xr:uid="{F9FEE340-9F19-44A0-8604-487DEB3377ED}">
+      <formula1>"Left,Right"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update 4/8/2026, Add Francken model and bug fix
</commit_message>
<xml_diff>
--- a/example/Excel Template for HWTT.xlsx
+++ b/example/Excel Template for HWTT.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usdot-my.sharepoint.com/personal/farhad_abdollahi_ctr_ad_dot_gov/Documents/GitHub_HWTT_Analysis_Tool/HWTT_Analysis_Tool/example/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usdot-my.sharepoint.com/personal/farhad_abdollahi_ctr_ad_dot_gov/Documents/GitHub_Projects/AutoHWTT/AutoHWTT_SourceCode/example/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="40" documentId="8_{BD69BDA0-91AA-41A6-AFBF-747FADBB4C07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FDEAD05F-A961-448D-A40D-193EAF34B7DA}"/>
@@ -396,14 +396,10 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -441,7 +437,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -547,7 +543,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -689,7 +685,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>

</xml_diff>